<commit_message>
analysis: IEEE-ready grayscale figures in English, Godot OOP 3rd run added
- benchmarkresults.xlsx: godot-oop-3 sheet added (was missing, now 3/3 runs)
- analyze.py: all labels translated to English; styling switched from
  color-coded lines to grayscale-safe distinct linestyles/markers (and
  hatch patterns for bar chart) so figures stay legible in B/W print
- figures exported as both PNG (300dpi) and PDF (vector, for LaTeX)

https://claude.ai/code/session_012BTzpM735GCUygYkiBMsKx
</commit_message>
<xml_diff>
--- a/results/benchmarks/benchmarkresults.xlsx
+++ b/results/benchmarks/benchmarkresults.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9084" firstSheet="4" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9084" firstSheet="5" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="unity-oop-1" sheetId="2" r:id="rId1"/>
@@ -20,17 +20,19 @@
     <sheet name="unity-dod-3" sheetId="7" r:id="rId6"/>
     <sheet name="godot-oop-1" sheetId="9" r:id="rId7"/>
     <sheet name="godot-oop-2" sheetId="10" r:id="rId8"/>
-    <sheet name="godot-dod-1" sheetId="12" r:id="rId9"/>
-    <sheet name="godot-dod-2" sheetId="13" r:id="rId10"/>
-    <sheet name="godot-dod-3" sheetId="14" r:id="rId11"/>
-    <sheet name="Sayfa1" sheetId="1" r:id="rId12"/>
+    <sheet name="godot-oop-3" sheetId="15" r:id="rId9"/>
+    <sheet name="godot-dod-1" sheetId="12" r:id="rId10"/>
+    <sheet name="godot-dod-2" sheetId="13" r:id="rId11"/>
+    <sheet name="godot-dod-3" sheetId="14" r:id="rId12"/>
+    <sheet name="Sayfa1" sheetId="1" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="benchmark_godot_dod_native_2026_06_16_22_27_58" localSheetId="10">'godot-dod-3'!$A$1:$J$6</definedName>
-    <definedName name="benchmark_godot_dod_native_2026_06_16_22_30_25" localSheetId="9">'godot-dod-2'!$A$1:$J$6</definedName>
-    <definedName name="benchmark_godot_dod_native_2026_06_16_22_33_11" localSheetId="8">'godot-dod-1'!$A$1:$J$6</definedName>
+    <definedName name="benchmark_godot_dod_native_2026_06_16_22_27_58" localSheetId="11">'godot-dod-3'!$A$1:$J$6</definedName>
+    <definedName name="benchmark_godot_dod_native_2026_06_16_22_30_25" localSheetId="10">'godot-dod-2'!$A$1:$J$6</definedName>
+    <definedName name="benchmark_godot_dod_native_2026_06_16_22_33_11" localSheetId="9">'godot-dod-1'!$A$1:$J$6</definedName>
     <definedName name="benchmark_godot_oop_2026_06_16_22_14_11" localSheetId="6">'godot-oop-1'!$A$1:$J$6</definedName>
     <definedName name="benchmark_godot_oop_2026_06_16_22_18_46" localSheetId="7">'godot-oop-2'!$A$1:$J$6</definedName>
+    <definedName name="benchmark_godot_oop_2026_06_16_23_20_14" localSheetId="8">'godot-oop-3'!$A$1:$J$6</definedName>
     <definedName name="benchmark_unity_dots_2026_06_16_21_33_10" localSheetId="5">'unity-dod-3'!$A$1:$J$6</definedName>
     <definedName name="benchmark_unity_dots_2026_06_16_21_40_11" localSheetId="4">'unity-dod-2'!$A$1:$J$6</definedName>
     <definedName name="benchmark_unity_dots_2026_06_16_22_09_27" localSheetId="3">'unity-dod-1'!$A$1:$J$6</definedName>
@@ -129,8 +131,8 @@
       </textFields>
     </textPr>
   </connection>
-  <connection id="6" name="benchmark_unity_dots_2026-06-16_21-33-10" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_dots_2026-06-16_21-33-10.csv" decimal="," thousands="." tab="0" comma="1">
+  <connection id="6" name="benchmark_godot_oop_2026-06-16_23-20-14" type="6" refreshedVersion="6" background="1" saveData="1">
+    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_godot_oop_2026-06-16_23-20-14.csv" decimal="," thousands="." tab="0" comma="1">
       <textFields count="10">
         <textField type="text"/>
         <textField type="text"/>
@@ -145,8 +147,8 @@
       </textFields>
     </textPr>
   </connection>
-  <connection id="7" name="benchmark_unity_dots_2026-06-16_21-40-11" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_dots_2026-06-16_21-40-11.csv" decimal="," thousands="." tab="0" comma="1">
+  <connection id="7" name="benchmark_unity_dots_2026-06-16_21-33-10" type="6" refreshedVersion="6" background="1" saveData="1">
+    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_dots_2026-06-16_21-33-10.csv" decimal="," thousands="." tab="0" comma="1">
       <textFields count="10">
         <textField type="text"/>
         <textField type="text"/>
@@ -161,8 +163,8 @@
       </textFields>
     </textPr>
   </connection>
-  <connection id="8" name="benchmark_unity_dots_2026-06-16_22-09-27" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_dots_2026-06-16_22-09-27.csv" decimal="," thousands="." tab="0" comma="1">
+  <connection id="8" name="benchmark_unity_dots_2026-06-16_21-40-11" type="6" refreshedVersion="6" background="1" saveData="1">
+    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_dots_2026-06-16_21-40-11.csv" decimal="," thousands="." tab="0" comma="1">
       <textFields count="10">
         <textField type="text"/>
         <textField type="text"/>
@@ -177,8 +179,8 @@
       </textFields>
     </textPr>
   </connection>
-  <connection id="9" name="benchmark_unity_oop_2026-06-16_20-37-54" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_oop_2026-06-16_20-37-54.csv" decimal="," thousands="." tab="0" comma="1">
+  <connection id="9" name="benchmark_unity_dots_2026-06-16_22-09-27" type="6" refreshedVersion="6" background="1" saveData="1">
+    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_dots_2026-06-16_22-09-27.csv" decimal="," thousands="." tab="0" comma="1">
       <textFields count="10">
         <textField type="text"/>
         <textField type="text"/>
@@ -193,8 +195,8 @@
       </textFields>
     </textPr>
   </connection>
-  <connection id="10" name="benchmark_unity_oop_2026-06-16_20-40-18" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_oop_2026-06-16_20-40-18.csv" decimal="," thousands="." tab="0" comma="1">
+  <connection id="10" name="benchmark_unity_oop_2026-06-16_20-37-54" type="6" refreshedVersion="6" background="1" saveData="1">
+    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_oop_2026-06-16_20-37-54.csv" decimal="," thousands="." tab="0" comma="1">
       <textFields count="10">
         <textField type="text"/>
         <textField type="text"/>
@@ -209,7 +211,23 @@
       </textFields>
     </textPr>
   </connection>
-  <connection id="11" name="benchmark_unity_oop_2026-06-16_20-42-52" type="6" refreshedVersion="6" background="1" saveData="1">
+  <connection id="11" name="benchmark_unity_oop_2026-06-16_20-40-18" type="6" refreshedVersion="6" background="1" saveData="1">
+    <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_oop_2026-06-16_20-40-18.csv" decimal="," thousands="." tab="0" comma="1">
+      <textFields count="10">
+        <textField type="text"/>
+        <textField type="text"/>
+        <textField type="text"/>
+        <textField type="text"/>
+        <textField type="text"/>
+        <textField type="text"/>
+        <textField type="text"/>
+        <textField type="text"/>
+        <textField type="text"/>
+        <textField type="text"/>
+      </textFields>
+    </textPr>
+  </connection>
+  <connection id="12" name="benchmark_unity_oop_2026-06-16_20-42-52" type="6" refreshedVersion="6" background="1" saveData="1">
     <textPr codePage="857" sourceFile="C:\Users\Emre\Desktop\results\benchmark_unity_oop_2026-06-16_20-42-52.csv" decimal="," thousands="." tab="0" comma="1">
       <textFields count="10">
         <textField type="text"/>
@@ -229,7 +247,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="447">
   <si>
     <t>EntityCount</t>
   </si>
@@ -1474,6 +1492,102 @@
   </si>
   <si>
     <t>3071</t>
+  </si>
+  <si>
+    <t>1.303</t>
+  </si>
+  <si>
+    <t>1.176</t>
+  </si>
+  <si>
+    <t>1.886</t>
+  </si>
+  <si>
+    <t>767.6</t>
+  </si>
+  <si>
+    <t>530.3</t>
+  </si>
+  <si>
+    <t>7677</t>
+  </si>
+  <si>
+    <t>5.996</t>
+  </si>
+  <si>
+    <t>5.558</t>
+  </si>
+  <si>
+    <t>6.841</t>
+  </si>
+  <si>
+    <t>0.104</t>
+  </si>
+  <si>
+    <t>166.8</t>
+  </si>
+  <si>
+    <t>146.2</t>
+  </si>
+  <si>
+    <t>1668</t>
+  </si>
+  <si>
+    <t>12.241</t>
+  </si>
+  <si>
+    <t>11.811</t>
+  </si>
+  <si>
+    <t>12.532</t>
+  </si>
+  <si>
+    <t>0.180</t>
+  </si>
+  <si>
+    <t>81.7</t>
+  </si>
+  <si>
+    <t>79.8</t>
+  </si>
+  <si>
+    <t>818</t>
+  </si>
+  <si>
+    <t>60.623</t>
+  </si>
+  <si>
+    <t>59.970</t>
+  </si>
+  <si>
+    <t>62.959</t>
+  </si>
+  <si>
+    <t>0.585</t>
+  </si>
+  <si>
+    <t>16.5</t>
+  </si>
+  <si>
+    <t>15.9</t>
+  </si>
+  <si>
+    <t>166</t>
+  </si>
+  <si>
+    <t>121.659</t>
+  </si>
+  <si>
+    <t>120.352</t>
+  </si>
+  <si>
+    <t>123.372</t>
+  </si>
+  <si>
+    <t>0.557</t>
+  </si>
+  <si>
+    <t>83</t>
   </si>
 </sst>
 </file>
@@ -1531,35 +1645,39 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_oop_2026-06-16_20-42-52" connectionId="11" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_oop_2026-06-16_20-42-52" connectionId="12" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable10.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_godot_dod_native_2026-06-16_22-33-11" connectionId="3" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable11.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_godot_dod_native_2026-06-16_22-30-25" connectionId="2" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
-<file path=xl/queryTables/queryTable11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/queryTables/queryTable12.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_godot_dod_native_2026-06-16_22-27-58" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_oop_2026-06-16_20-40-18" connectionId="10" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_oop_2026-06-16_20-40-18" connectionId="11" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_oop_2026-06-16_20-37-54" connectionId="9" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_oop_2026-06-16_20-37-54" connectionId="10" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_dots_2026-06-16_22-09-27" connectionId="8" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_dots_2026-06-16_22-09-27" connectionId="9" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_dots_2026-06-16_21-40-11" connectionId="7" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_dots_2026-06-16_21-40-11" connectionId="8" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_dots_2026-06-16_21-33-10" connectionId="6" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_unity_dots_2026-06-16_21-33-10" connectionId="7" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable7.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1571,7 +1689,7 @@
 </file>
 
 <file path=xl/queryTables/queryTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_godot_dod_native_2026-06-16_22-33-11" connectionId="3" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="benchmark_godot_oop_2026-06-16_23-20-14" connectionId="6" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2103,28 +2221,28 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>359</v>
+        <v>322</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>360</v>
+        <v>323</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>12</v>
+        <v>324</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>361</v>
+        <v>325</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>362</v>
+        <v>326</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>363</v>
+        <v>327</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>328</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>364</v>
+        <v>329</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>19</v>
@@ -2135,19 +2253,19 @@
         <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>365</v>
+        <v>330</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>366</v>
+        <v>331</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>332</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>367</v>
+        <v>333</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>368</v>
+        <v>334</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>335</v>
@@ -2156,7 +2274,7 @@
         <v>336</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>369</v>
+        <v>337</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>19</v>
@@ -2170,16 +2288,16 @@
         <v>338</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>370</v>
+        <v>339</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>332</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>371</v>
+        <v>340</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>372</v>
+        <v>341</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>335</v>
@@ -2188,7 +2306,7 @@
         <v>342</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>373</v>
+        <v>343</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>19</v>
@@ -2199,28 +2317,28 @@
         <v>38</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>374</v>
+        <v>344</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>236</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>375</v>
+        <v>345</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>250</v>
+        <v>346</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>376</v>
+        <v>347</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>377</v>
+        <v>348</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>349</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>378</v>
+        <v>350</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>19</v>
@@ -2231,28 +2349,28 @@
         <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>379</v>
+        <v>351</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>380</v>
+        <v>352</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>381</v>
+        <v>353</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>325</v>
+        <v>354</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>382</v>
+        <v>355</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>383</v>
+        <v>356</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>357</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>384</v>
+        <v>358</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>19</v>
@@ -2317,28 +2435,28 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>385</v>
+        <v>359</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>386</v>
+        <v>360</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>387</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>388</v>
+        <v>361</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>389</v>
+        <v>362</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>390</v>
+        <v>363</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>391</v>
+        <v>328</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>392</v>
+        <v>364</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>19</v>
@@ -2352,25 +2470,25 @@
         <v>365</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>393</v>
+        <v>366</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>332</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>367</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>395</v>
+        <v>368</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>335</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>396</v>
+        <v>336</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>397</v>
+        <v>369</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>19</v>
@@ -2381,19 +2499,19 @@
         <v>29</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>398</v>
+        <v>338</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>399</v>
+        <v>370</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>332</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>400</v>
+        <v>371</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>401</v>
+        <v>372</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>335</v>
@@ -2402,7 +2520,7 @@
         <v>342</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>402</v>
+        <v>373</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>19</v>
@@ -2413,28 +2531,28 @@
         <v>38</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>403</v>
+        <v>374</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>236</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>404</v>
+        <v>375</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>405</v>
+        <v>250</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>406</v>
+        <v>376</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>407</v>
+        <v>377</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>349</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>408</v>
+        <v>378</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>19</v>
@@ -2445,28 +2563,28 @@
         <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>409</v>
+        <v>379</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>410</v>
+        <v>380</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>411</v>
+        <v>381</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>354</v>
+        <v>325</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>412</v>
+        <v>382</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>413</v>
+        <v>383</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>357</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>414</v>
+        <v>384</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>19</v>
@@ -2478,6 +2596,220 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4038,28 +4370,28 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>322</v>
+        <v>415</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>323</v>
+        <v>416</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>324</v>
+        <v>417</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>325</v>
+        <v>250</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>326</v>
+        <v>418</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>327</v>
+        <v>419</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>328</v>
+        <v>264</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>329</v>
+        <v>420</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>19</v>
@@ -4070,28 +4402,28 @@
         <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>330</v>
+        <v>421</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>331</v>
+        <v>422</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>332</v>
+        <v>423</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>333</v>
+        <v>424</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>334</v>
+        <v>425</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>335</v>
+        <v>426</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>336</v>
+        <v>272</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>337</v>
+        <v>427</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>19</v>
@@ -4102,28 +4434,28 @@
         <v>29</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>338</v>
+        <v>428</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>339</v>
+        <v>429</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>332</v>
+        <v>430</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>340</v>
+        <v>431</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>341</v>
+        <v>432</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>335</v>
+        <v>433</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>342</v>
+        <v>280</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>343</v>
+        <v>434</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>19</v>
@@ -4134,28 +4466,28 @@
         <v>38</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>344</v>
+        <v>435</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>236</v>
+        <v>436</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>345</v>
+        <v>437</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>346</v>
+        <v>438</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>347</v>
+        <v>439</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>348</v>
+        <v>440</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>349</v>
+        <v>288</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>350</v>
+        <v>441</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>19</v>
@@ -4166,28 +4498,28 @@
         <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>351</v>
+        <v>442</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>352</v>
+        <v>443</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>353</v>
+        <v>444</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>354</v>
+        <v>445</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>355</v>
+        <v>321</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>356</v>
+        <v>295</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>357</v>
+        <v>296</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>358</v>
+        <v>446</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>19</v>

</xml_diff>